<commit_message>
update table 1 results
</commit_message>
<xml_diff>
--- a/OMOP Analysis/Results/Cohort/Table1_OMOP.xlsx
+++ b/OMOP Analysis/Results/Cohort/Table1_OMOP.xlsx
@@ -357,31 +357,31 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>**Characteristic**</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>**N = 23,386**</t>
+          <t>N = 22,900</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Age at fracture occurrence</t>
+          <t>Age at Fracture Occurrence</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>70 (61, 81)</t>
+          <t>71 (61, 81)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fracture site</t>
+          <t>Fracture fracture_site</t>
         </is>
       </c>
     </row>
@@ -393,7 +393,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3,173 (14%)</t>
+          <t>3,197 (14%)</t>
         </is>
       </c>
     </row>
@@ -405,7 +405,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,682 (7.2%)</t>
+          <t>1,699 (7.4%)</t>
         </is>
       </c>
     </row>
@@ -417,129 +417,129 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18,531 (79%)</t>
+          <t>18,004 (79%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Censoring event</t>
+          <t>Censoring Event</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cancer</t>
+          <t>Max of 730 days from index date</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>745 (3.2%)</t>
+          <t>9,730 (42%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cancer, Fracture ensuing incident (index) fracture</t>
+          <t>End of Study</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2 (&lt;0.1%)</t>
+          <t>6,026 (26%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cancer, Paget’s disease of the bone, or other metabolic bone diseases</t>
+          <t>Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>4,071 (18%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Death</t>
+          <t>End of data collection period</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1,266 (5.4%)</t>
+          <t>1,479 (6.5%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>End of data collection period</t>
+          <t>Death</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1,838 (7.9%)</t>
+          <t>1,150 (5.0%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>End of data collection period, Cancer</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>379 (1.7%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>End of data collection period, Fracture ensuing incident (index) fracture</t>
+          <t>Paget’s disease of the bone, or other metabolic bone diseases</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2 (&lt;0.1%)</t>
+          <t>54 (0.2%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fracture ensuing incident (index) fracture</t>
+          <t>Max of 730 days from index date, End of Study</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4,036 (17%)</t>
+          <t>7 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date</t>
+          <t>Cancer, Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>15,411 (66%)</t>
+          <t>1 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, Cancer</t>
+          <t>End of data collection period, Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -551,12 +551,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, End of data collection period</t>
+          <t>Fracture ensuing incident (index) fracture, End of Study</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2 (&lt;0.1%)</t>
+          <t>1 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
@@ -575,48 +575,43 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, Paget’s disease of the bone, or other metabolic bone diseases</t>
+          <t>Follow up time</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>578 (192, 730)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Paget’s disease of the bone, or other metabolic bone diseases</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>78 (0.3%)</t>
+          <t>Heathcare Service User Status</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Paget’s disease of the bone, or other metabolic bone diseases, Fracture ensuing incident (index) fracture</t>
+          <t>Non-User</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>682 (3.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Follow up time</t>
+          <t>User</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>730 (365, 730)</t>
+          <t>22,218 (97%)</t>
         </is>
       </c>
     </row>

</xml_diff>